<commit_message>
Back to orig with Utopia
</commit_message>
<xml_diff>
--- a/mosip_master/xlsx/identity_schema.xlsx
+++ b/mosip_master/xlsx/identity_schema.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BarnabyTwyford\repos\mosip-data\mosip_master\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project\Mosip\mosip-data\mosip_master\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4499C40-F346-4BCA-9E39-79EEA3CBBEC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E632B33-EFBA-45CC-B1A2-807AF397E164}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -406,7 +406,19 @@
 					"fieldType": "default"
 				},
 				"individualAuthBiometrics": {
-					"bioAttributes": [						
+					"bioAttributes": [
+						"leftEye",
+						"rightEye",
+						"rightIndex",
+						"rightLittle",
+						"rightRing",
+						"rightMiddle",
+						"leftIndex",
+						"leftLittle",
+						"leftRing",
+						"leftMiddle",
+						"leftThumb",
+						"rightThumb",
 						"face"
 					],
 					"fieldCategory": "pvt",
@@ -955,23 +967,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AMJ3"/>
-  <sheetFormatPr defaultColWidth="8.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.42578125" style="1"/>
-    <col min="2" max="2" width="8.42578125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="11.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="8.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="8.453125" style="1"/>
+    <col min="2" max="2" width="8.453125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="11.54296875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="8.453125" style="1" customWidth="1"/>
     <col min="5" max="5" width="31" style="1" customWidth="1"/>
-    <col min="6" max="6" width="53.7109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="13.42578125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="53.7265625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7265625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13.453125" style="2" customWidth="1"/>
     <col min="9" max="9" width="10" style="1" customWidth="1"/>
-    <col min="10" max="10" width="8.42578125" style="2"/>
-    <col min="11" max="1023" width="8.42578125" style="1"/>
-    <col min="1024" max="1024" width="11.5703125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="8.453125" style="2"/>
+    <col min="11" max="1023" width="8.453125" style="1"/>
+    <col min="1024" max="1024" width="11.54296875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1003,7 +1015,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -1035,7 +1047,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B3" s="1"/>
       <c r="F3" s="5"/>
     </row>

</xml_diff>